<commit_message>
docs: Sydney's answers for notecards 16-21
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Notecards-Need-Your-Input.xlsx
+++ b/docs/Notecards-Need-Your-Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830BF44D-40F4-A34F-85A8-EA53E854ABD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F792DF-7247-CE4D-A382-1248C0CB104B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="128">
   <si>
     <t>How to fill this in: click the link to open the card on your current site, look at its personalization section, then type its questions in "Your answer" (e.g. "Boots color: brown / black; Hat placement: top or bottom"). Write "standard" if it only needs Text, Font, Text Color and return address. Leave a row blank if unsure.</t>
   </si>
@@ -392,6 +392,24 @@
   </si>
   <si>
     <t>name, font, text color, image location, name &amp; return address</t>
+  </si>
+  <si>
+    <t>no changes</t>
+  </si>
+  <si>
+    <t>name, font, text color, color for medical icon, name and return address</t>
+  </si>
+  <si>
+    <t>name, font, color for text, border color, color for pom pom, color for megaphone, name &amp; return address</t>
+  </si>
+  <si>
+    <t>university/school name, class year, name, outer border color, inner border color, text color, any additional instructions, name &amp; return address</t>
+  </si>
+  <si>
+    <t>no changes from current website</t>
+  </si>
+  <si>
+    <t>no chnages from current website</t>
   </si>
 </sst>
 </file>
@@ -411,12 +429,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF1450A0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -810,7 +830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1090,7 +1110,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1126,9 +1146,11 @@
       <c r="E18" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F18" s="4"/>
-    </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="F18" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1144,7 +1166,9 @@
       <c r="E19" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F19" s="4"/>
+      <c r="F19" s="4" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
@@ -1162,9 +1186,11 @@
       <c r="E20" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="F20" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1180,7 +1206,9 @@
       <c r="E21" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F21" s="4"/>
+      <c r="F21" s="4" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
@@ -1198,7 +1226,9 @@
       <c r="E22" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
@@ -1216,9 +1246,11 @@
       <c r="E23" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F23" s="4"/>
-    </row>
-    <row r="24" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="F23" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1254,7 +1286,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1272,7 +1304,7 @@
       </c>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1290,7 +1322,7 @@
       </c>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1308,7 +1340,7 @@
       </c>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1326,7 +1358,7 @@
       </c>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1416,7 +1448,7 @@
       </c>
       <c r="F34" s="4"/>
     </row>
-    <row r="35" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -1488,7 +1520,7 @@
       </c>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -1524,7 +1556,7 @@
       </c>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -1560,7 +1592,7 @@
       </c>
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -1596,7 +1628,7 @@
       </c>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -1614,7 +1646,7 @@
       </c>
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>44</v>
       </c>

</xml_diff>

<commit_message>
docs: Sydney's answers for notecards 22-44
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Notecards-Need-Your-Input.xlsx
+++ b/docs/Notecards-Need-Your-Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F792DF-7247-CE4D-A382-1248C0CB104B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954D1F11-78C4-1D45-8A44-2D123C1D94B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="142">
   <si>
     <t>How to fill this in: click the link to open the card on your current site, look at its personalization section, then type its questions in "Your answer" (e.g. "Boots color: brown / black; Hat placement: top or bottom"). Write "standard" if it only needs Text, Font, Text Color and return address. Leave a row blank if unsure.</t>
   </si>
@@ -410,6 +410,48 @@
   </si>
   <si>
     <t>no chnages from current website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name, text color, font, gymnast color, name and address </t>
+  </si>
+  <si>
+    <t>name, font, text color, name and address</t>
+  </si>
+  <si>
+    <t>name, return &amp; adddress</t>
+  </si>
+  <si>
+    <t>name, font, text color, orange placement: top center, bottom left, name &amp; return address</t>
+  </si>
+  <si>
+    <t>name, font, text color, pelican placement: top center or bottom right, name &amp; return address</t>
+  </si>
+  <si>
+    <t>name, font, text color, snowboarder color, name &amp; return address</t>
+  </si>
+  <si>
+    <t>name, font, text color, name &amp; address</t>
+  </si>
+  <si>
+    <t>duplicate listing - delete listing.</t>
+  </si>
+  <si>
+    <t>same as shown. Rank insignia free text is correct</t>
+  </si>
+  <si>
+    <t>name, font, text color, wren location: top center, bottom left, name &amp; address</t>
+  </si>
+  <si>
+    <t>name, font, text color, paddle color, paddle color: top center, bottom left, name &amp; return address</t>
+  </si>
+  <si>
+    <t>delete listing, duplicate.</t>
+  </si>
+  <si>
+    <t>name, text color, name &amp; address</t>
+  </si>
+  <si>
+    <t>name, text color, name &amp; return address</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1308,9 @@
       <c r="E24" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F24" s="4"/>
+      <c r="F24" s="4" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
@@ -1284,7 +1328,9 @@
       <c r="E25" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
@@ -1302,7 +1348,9 @@
       <c r="E26" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F26" s="4"/>
+      <c r="F26" s="4" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
@@ -1320,7 +1368,9 @@
       <c r="E27" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F27" s="4"/>
+      <c r="F27" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
@@ -1338,7 +1388,9 @@
       <c r="E28" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F28" s="4"/>
+      <c r="F28" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
@@ -1356,7 +1408,9 @@
       <c r="E29" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F29" s="4"/>
+      <c r="F29" s="4" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
@@ -1374,7 +1428,9 @@
       <c r="E30" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F30" s="4"/>
+      <c r="F30" s="4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
@@ -1392,7 +1448,9 @@
       <c r="E31" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F31" s="4"/>
+      <c r="F31" s="4" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
@@ -1410,7 +1468,9 @@
       <c r="E32" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F32" s="4"/>
+      <c r="F32" s="4" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="33" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
@@ -1428,9 +1488,11 @@
       <c r="E33" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F33" s="4"/>
-    </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="F33" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -1446,7 +1508,9 @@
       <c r="E34" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F34" s="4"/>
+      <c r="F34" s="4" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
@@ -1482,7 +1546,9 @@
       <c r="E36" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F36" s="4"/>
+      <c r="F36" s="4" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="37" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
@@ -1500,7 +1566,9 @@
       <c r="E37" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F37" s="4"/>
+      <c r="F37" s="4" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="38" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
@@ -1518,7 +1586,9 @@
       <c r="E38" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F38" s="4"/>
+      <c r="F38" s="4" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="39" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
@@ -1536,9 +1606,11 @@
       <c r="E39" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="4"/>
-    </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="F39" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -1554,7 +1626,9 @@
       <c r="E40" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F40" s="4"/>
+      <c r="F40" s="4" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
@@ -1572,7 +1646,9 @@
       <c r="E41" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="4"/>
+      <c r="F41" s="4" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="42" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
@@ -1590,7 +1666,9 @@
       <c r="E42" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F42" s="4"/>
+      <c r="F42" s="4" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="43" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
@@ -1608,7 +1686,9 @@
       <c r="E43" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F43" s="4"/>
+      <c r="F43" s="4" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="44" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
@@ -1626,7 +1706,9 @@
       <c r="E44" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="F44" s="4"/>
+      <c r="F44" s="4" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="45" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
@@ -1644,7 +1726,9 @@
       <c r="E45" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F45" s="4"/>
+      <c r="F45" s="4" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="46" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
@@ -1662,7 +1746,9 @@
       <c r="E46" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F46" s="4"/>
+      <c r="F46" s="4" t="s">
+        <v>139</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>